<commit_message>
Actualizacion matriz entrenamiento modelo
Se realiza ajustes a umbrales de acuerdo a datos sisnteticos para definicion de matriz logica para entrenamiento de modelo
</commit_message>
<xml_diff>
--- a/Matriz_Logica_EnergiAI_Teams_72.xlsx
+++ b/Matriz_Logica_EnergiAI_Teams_72.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Estudios Vigentes\ESPECIALIZACION DATA SCIENCE ALURA ORACLE\Hackathon G9 Equipo 72\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Estudios Vigentes\ESPECIALIZACION DATA SCIENCE ALURA ORACLE\Hackathon G9 Equipo 72\Data Science Plan A\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755" tabRatio="857"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755" tabRatio="857" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="matriz_logica" sheetId="7" r:id="rId1"/>
+    <sheet name="matriz_logica V1" sheetId="7" r:id="rId1"/>
+    <sheet name="matriz_logica V2" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511" iterateDelta="1E-4"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="68">
   <si>
     <t>Perfil Calculado</t>
   </si>
@@ -216,6 +217,18 @@
   </si>
   <si>
     <t>Auditoría de Empaques: Revise el sellado hermético de las gomas (burletes) de las puertas de refrigeración. Si el consumo nocturno no baja, los equipos están perdiendo frío continuamente.</t>
+  </si>
+  <si>
+    <t>Eficiente  (&lt; 8.29) | Moderado (8.29 - 11.78) | Ineficiente (&gt; 11.78)</t>
+  </si>
+  <si>
+    <t>Eficiente  (&lt; 3.14) | Moderado (3.14 - 5.02) | Ineficiente (&gt; 5.02)</t>
+  </si>
+  <si>
+    <t>Eficiente (&lt; 19.56) | Moderado (19.56 - 27.49) | Ineficiente (&gt; 27.49)</t>
+  </si>
+  <si>
+    <t>Eficiente (&lt; 27.14) | Moderado (27.14 - 38.98) | Ineficiente (&gt; 38.98)</t>
   </si>
 </sst>
 </file>
@@ -935,4 +948,376 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="164.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>